<commit_message>
Update corrected GDSC drug class workbook
</commit_message>
<xml_diff>
--- a/Code/gdsc_ploidy_analysis/data/manual/drug_class_final_used_with_primary_secondary_corrected.xlsx
+++ b/Code/gdsc_ploidy_analysis/data/manual/drug_class_final_used_with_primary_secondary_corrected.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/4470246/Repositories/Gemcitabine-model/Code/gdsc_ploidy_analysis/data/manual/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/4475916/Repositories/Gemcitabine-model/Code/gdsc_ploidy_analysis/data/manual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91FB0D1C-DCE9-0F4B-ADF6-6AA1C1C1680D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B848E51F-FE0C-B649-BF74-7C15CD0710E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4580" yWindow="-24400" windowWidth="34560" windowHeight="21580" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="drug_class_final_used_with_prim" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9063" uniqueCount="1966">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9065" uniqueCount="1966">
   <si>
     <t>primary_anticancer_class</t>
   </si>
@@ -5918,7 +5918,7 @@
     <t>Kinase inhibitors</t>
   </si>
   <si>
-    <t>DNA damage and repair agents</t>
+    <t>Chemotherapy agents</t>
   </si>
 </sst>
 </file>
@@ -40095,9 +40095,7 @@
       <c r="B6">
         <v>19</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>1965</v>
-      </c>
+      <c r="C6" s="1"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -40144,6 +40142,9 @@
       <c r="B11">
         <v>8</v>
       </c>
+      <c r="C11" t="s">
+        <v>1965</v>
+      </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -40163,7 +40164,7 @@
       <c r="B13">
         <v>8</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>1965</v>
       </c>
     </row>
@@ -40174,7 +40175,7 @@
       <c r="B14">
         <v>6</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>1965</v>
       </c>
     </row>
@@ -40185,6 +40186,9 @@
       <c r="B15">
         <v>6</v>
       </c>
+      <c r="C15" t="s">
+        <v>1965</v>
+      </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -40208,6 +40212,9 @@
       </c>
       <c r="B18">
         <v>3</v>
+      </c>
+      <c r="C18" t="s">
+        <v>1965</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>